<commit_message>
Harden pricing build and publish Newton designs
</commit_message>
<xml_diff>
--- a/private-source/price-lists/Lookup.xlsx
+++ b/private-source/price-lists/Lookup.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimday/Library/CloudStorage/OneDrive-pacificartisanlabs.com/Report Data/Reference Files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimday/Documents/GitHub/artisan-site/private-source/price-lists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24D94CD4-1258-FB47-A9D5-F14CF6D978E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E3D2B911-C083-D443-B159-ED4BC837BA46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19320" yWindow="4320" windowWidth="28800" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="38120" windowHeight="13160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Export" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Export!$A$1:$F$556</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Export!$A$1:$F$522</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2827" uniqueCount="764">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2827" uniqueCount="768">
   <si>
     <t>lenstyle</t>
   </si>
@@ -2169,10 +2169,46 @@
     <t>Generic</t>
   </si>
   <si>
+    <t>SEQUEL MEETING</t>
+  </si>
+  <si>
+    <t>SEQUEL *</t>
+  </si>
+  <si>
     <t>SEQUEL PAL *</t>
   </si>
   <si>
-    <t>SEQUEL *</t>
+    <t>CD DIGITAL RD*</t>
+  </si>
+  <si>
+    <t>SD CONCEPT *</t>
+  </si>
+  <si>
+    <t>SD REACH *</t>
+  </si>
+  <si>
+    <t>SYNC III *</t>
+  </si>
+  <si>
+    <t>EYEZEN+ *</t>
+  </si>
+  <si>
+    <t>ARRAY *</t>
+  </si>
+  <si>
+    <t>ARRAY W *</t>
+  </si>
+  <si>
+    <t>ARRAY 2 *</t>
+  </si>
+  <si>
+    <t>ARRAY 2 W *</t>
+  </si>
+  <si>
+    <t>ENDLSS OFF *</t>
+  </si>
+  <si>
+    <t>ENDLESS PLUS *</t>
   </si>
   <si>
     <t>AUTO II ATT *</t>
@@ -2181,154 +2217,130 @@
     <t>Autograph 2 Attitude</t>
   </si>
   <si>
+    <t>AUTO II+ *</t>
+  </si>
+  <si>
+    <t>AUTO II *</t>
+  </si>
+  <si>
+    <t>AUTO III *</t>
+  </si>
+  <si>
+    <t>INTOUCH *</t>
+  </si>
+  <si>
     <t>SPECTRUM *</t>
   </si>
   <si>
-    <t>AUTO II+ *</t>
-  </si>
-  <si>
-    <t>AUTO II *</t>
+    <t>SPECTRUM+ *</t>
+  </si>
+  <si>
+    <t>REST-W *</t>
+  </si>
+  <si>
+    <t>TOKAI AS SV *</t>
+  </si>
+  <si>
+    <t>AS SV</t>
+  </si>
+  <si>
+    <t>Bi-AS *</t>
+  </si>
+  <si>
+    <t>Bi-AS</t>
+  </si>
+  <si>
+    <t>Bi-AS C</t>
+  </si>
+  <si>
+    <t>Bi-AS S</t>
+  </si>
+  <si>
+    <t>TOKAI EASYONE *</t>
+  </si>
+  <si>
+    <t>Easyone</t>
+  </si>
+  <si>
+    <t>TS 5X HM LG</t>
+  </si>
+  <si>
+    <t>TS 5X HM LG *</t>
+  </si>
+  <si>
+    <t>TS 5X TW</t>
+  </si>
+  <si>
+    <t>TS 5X TW *</t>
+  </si>
+  <si>
+    <t>TS 9X HM WD</t>
+  </si>
+  <si>
+    <t>TS 9X HM WD *</t>
+  </si>
+  <si>
+    <t>TS 9X TW</t>
+  </si>
+  <si>
+    <t>TS 9X TW *</t>
+  </si>
+  <si>
+    <t>ETHOS PLUS *</t>
   </si>
   <si>
     <t>Unity Relieve *</t>
   </si>
   <si>
-    <t>ARRAY W *</t>
-  </si>
-  <si>
-    <t>ARRAY *</t>
-  </si>
-  <si>
-    <t>TOKAI EASYONE *</t>
-  </si>
-  <si>
-    <t>Easyone</t>
-  </si>
-  <si>
-    <t>TOKAI AS SV *</t>
-  </si>
-  <si>
-    <t>AS SV</t>
-  </si>
-  <si>
-    <t>Bi-AS</t>
-  </si>
-  <si>
-    <t>Bi-AS S</t>
-  </si>
-  <si>
-    <t>Bi-AS C</t>
-  </si>
-  <si>
-    <t>Bi-AS *</t>
-  </si>
-  <si>
-    <t>REST-W *</t>
-  </si>
-  <si>
-    <t>SPECTRUM+ *</t>
-  </si>
-  <si>
-    <t>INTOUCH *</t>
-  </si>
-  <si>
-    <t>ARRAY 2 *</t>
-  </si>
-  <si>
-    <t>ARRAY 2 W *</t>
-  </si>
-  <si>
-    <t>EYEZEN+ *</t>
-  </si>
-  <si>
-    <t>SYNC III *</t>
-  </si>
-  <si>
-    <t>ENDLSS OFF *</t>
-  </si>
-  <si>
-    <t>SD REACH *</t>
-  </si>
-  <si>
-    <t>ENDLESS PLUS *</t>
-  </si>
-  <si>
-    <t>ETHOS PLUS *</t>
-  </si>
-  <si>
-    <t>SD CONCEPT *</t>
-  </si>
-  <si>
-    <t>AUTO III *</t>
+    <t>UNITY3 MOBILE</t>
+  </si>
+  <si>
+    <t>V3 Mobile</t>
+  </si>
+  <si>
+    <t>UNITY3 MOBILE *</t>
+  </si>
+  <si>
+    <t>VX X 4D</t>
+  </si>
+  <si>
+    <t>X Design 4D</t>
   </si>
   <si>
     <t>IDLS3 *</t>
   </si>
   <si>
+    <t>LS3 SUN * I</t>
+  </si>
+  <si>
     <t>IDLS3 * I</t>
   </si>
   <si>
     <t>IDLS3 *R</t>
   </si>
   <si>
-    <t>CD DIGITAL RD*</t>
-  </si>
-  <si>
     <t>IDLS3 *R I</t>
   </si>
   <si>
     <t>IDLS4 *</t>
   </si>
   <si>
+    <t>LS4 SUN*</t>
+  </si>
+  <si>
     <t>Largo WS *</t>
   </si>
   <si>
     <t>Largo WS</t>
   </si>
   <si>
-    <t>LS4 SUN*</t>
-  </si>
-  <si>
-    <t>LS3 SUN * I</t>
-  </si>
-  <si>
-    <t>TS 5X HM LG</t>
-  </si>
-  <si>
-    <t>TS 5X HM LG *</t>
-  </si>
-  <si>
-    <t>TS 5X TW</t>
-  </si>
-  <si>
-    <t>TS 5X TW *</t>
-  </si>
-  <si>
-    <t>TS 9X HM WD</t>
-  </si>
-  <si>
-    <t>TS 9X HM WD *</t>
-  </si>
-  <si>
-    <t>TS 9X TW</t>
-  </si>
-  <si>
-    <t>TS 9X TW *</t>
-  </si>
-  <si>
-    <t>UNITY3 MOBILE</t>
-  </si>
-  <si>
-    <t>UNITY3 MOBILE *</t>
-  </si>
-  <si>
-    <t>V3 Mobile</t>
-  </si>
-  <si>
-    <t>X Design 4D</t>
-  </si>
-  <si>
-    <t>VX X 4D</t>
+    <t>SEQUEL COMPUTER</t>
+  </si>
+  <si>
+    <t>Sequel Meeting</t>
+  </si>
+  <si>
+    <t>Sequel Computer</t>
   </si>
 </sst>
 </file>
@@ -2846,7 +2858,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>744</v>
+        <v>713</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>376</v>
@@ -4159,7 +4171,7 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
-        <v>739</v>
+        <v>714</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>419</v>
@@ -4299,7 +4311,7 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
-        <v>736</v>
+        <v>715</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>421</v>
@@ -5153,7 +5165,7 @@
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A125" s="2" t="s">
-        <v>734</v>
+        <v>716</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>705</v>
@@ -5424,7 +5436,7 @@
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139" s="2" t="s">
-        <v>733</v>
+        <v>717</v>
       </c>
       <c r="B139" t="s">
         <v>697</v>
@@ -5820,7 +5832,7 @@
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A160" s="2" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="B160" s="2" t="s">
         <v>361</v>
@@ -5840,7 +5852,7 @@
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A161" s="2" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B161" s="2" t="s">
         <v>361</v>
@@ -5957,7 +5969,7 @@
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A167" s="2" t="s">
-        <v>731</v>
+        <v>720</v>
       </c>
       <c r="B167" s="2" t="s">
         <v>362</v>
@@ -5977,7 +5989,7 @@
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A168" s="2" t="s">
-        <v>732</v>
+        <v>721</v>
       </c>
       <c r="B168" s="2" t="s">
         <v>362</v>
@@ -7909,7 +7921,7 @@
     </row>
     <row r="270" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A270" s="2" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="B270" s="2" t="s">
         <v>387</v>
@@ -8603,7 +8615,7 @@
     </row>
     <row r="305" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A305" s="2" t="s">
-        <v>737</v>
+        <v>723</v>
       </c>
       <c r="B305" s="2" t="s">
         <v>383</v>
@@ -9134,6 +9146,9 @@
       <c r="D331" s="2" t="s">
         <v>485</v>
       </c>
+      <c r="E331" s="2">
+        <v>4</v>
+      </c>
       <c r="F331" s="2" t="s">
         <v>700</v>
       </c>
@@ -9151,6 +9166,9 @@
       <c r="D332" t="s">
         <v>485</v>
       </c>
+      <c r="E332" s="2">
+        <v>4</v>
+      </c>
       <c r="F332" t="s">
         <v>700</v>
       </c>
@@ -9168,6 +9186,9 @@
       <c r="D333" s="2" t="s">
         <v>485</v>
       </c>
+      <c r="E333" s="2">
+        <v>4</v>
+      </c>
       <c r="F333" s="2" t="s">
         <v>700</v>
       </c>
@@ -9185,6 +9206,9 @@
       <c r="D334" t="s">
         <v>485</v>
       </c>
+      <c r="E334" s="2">
+        <v>4</v>
+      </c>
       <c r="F334" t="s">
         <v>700</v>
       </c>
@@ -9202,6 +9226,9 @@
       <c r="D335" t="s">
         <v>485</v>
       </c>
+      <c r="E335" s="2">
+        <v>4</v>
+      </c>
       <c r="F335" t="s">
         <v>700</v>
       </c>
@@ -9227,40 +9254,40 @@
       </c>
     </row>
     <row r="337" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A337" t="s">
-        <v>227</v>
+      <c r="A337" s="2" t="s">
+        <v>710</v>
       </c>
       <c r="B337" s="2" t="s">
-        <v>410</v>
-      </c>
-      <c r="C337" s="2" t="s">
-        <v>489</v>
-      </c>
-      <c r="D337" s="2" t="s">
-        <v>484</v>
-      </c>
-      <c r="E337" s="2">
-        <v>5</v>
-      </c>
-      <c r="F337" s="2" t="s">
+        <v>766</v>
+      </c>
+      <c r="C337" t="s">
+        <v>506</v>
+      </c>
+      <c r="D337" t="s">
+        <v>485</v>
+      </c>
+      <c r="E337">
+        <v>4</v>
+      </c>
+      <c r="F337" t="s">
         <v>700</v>
       </c>
     </row>
     <row r="338" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A338" t="s">
-        <v>496</v>
+      <c r="A338" s="2" t="s">
+        <v>765</v>
       </c>
       <c r="B338" s="2" t="s">
-        <v>410</v>
+        <v>767</v>
       </c>
       <c r="C338" s="2" t="s">
-        <v>488</v>
+        <v>506</v>
       </c>
       <c r="D338" s="2" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E338" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F338" s="2" t="s">
         <v>700</v>
@@ -9268,13 +9295,13 @@
     </row>
     <row r="339" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A339" t="s">
-        <v>497</v>
+        <v>227</v>
       </c>
       <c r="B339" s="2" t="s">
         <v>410</v>
       </c>
       <c r="C339" s="2" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="D339" s="2" t="s">
         <v>484</v>
@@ -9288,7 +9315,7 @@
     </row>
     <row r="340" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A340" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="B340" s="2" t="s">
         <v>410</v>
@@ -9308,19 +9335,19 @@
     </row>
     <row r="341" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A341" t="s">
-        <v>228</v>
+        <v>497</v>
       </c>
       <c r="B341" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C341" s="2" t="s">
-        <v>507</v>
+        <v>488</v>
       </c>
       <c r="D341" s="2" t="s">
-        <v>33</v>
+        <v>484</v>
       </c>
       <c r="E341" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F341" s="2" t="s">
         <v>700</v>
@@ -9328,16 +9355,19 @@
     </row>
     <row r="342" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A342" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B342" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C342" s="2" t="s">
-        <v>507</v>
+        <v>488</v>
       </c>
       <c r="D342" s="2" t="s">
-        <v>33</v>
+        <v>484</v>
+      </c>
+      <c r="E342" s="2">
+        <v>5</v>
       </c>
       <c r="F342" s="2" t="s">
         <v>700</v>
@@ -9345,67 +9375,79 @@
     </row>
     <row r="343" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A343" t="s">
-        <v>611</v>
-      </c>
-      <c r="B343" t="s">
-        <v>688</v>
-      </c>
-      <c r="C343" t="s">
+        <v>228</v>
+      </c>
+      <c r="B343" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="C343" s="2" t="s">
         <v>507</v>
       </c>
-      <c r="D343" t="s">
+      <c r="D343" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F343" t="s">
+      <c r="E343" s="2">
+        <v>1</v>
+      </c>
+      <c r="F343" s="2" t="s">
         <v>700</v>
       </c>
     </row>
     <row r="344" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A344" t="s">
-        <v>612</v>
-      </c>
-      <c r="B344" t="s">
-        <v>688</v>
-      </c>
-      <c r="C344" t="s">
+        <v>499</v>
+      </c>
+      <c r="B344" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="C344" s="2" t="s">
         <v>507</v>
       </c>
-      <c r="D344" t="s">
+      <c r="D344" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F344" t="s">
+      <c r="E344" s="2">
+        <v>1</v>
+      </c>
+      <c r="F344" s="2" t="s">
         <v>700</v>
       </c>
     </row>
     <row r="345" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A345" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="B345" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="C345" t="s">
-        <v>489</v>
+        <v>507</v>
       </c>
       <c r="D345" t="s">
-        <v>484</v>
+        <v>33</v>
+      </c>
+      <c r="E345" s="2">
+        <v>1</v>
       </c>
       <c r="F345" t="s">
         <v>700</v>
       </c>
     </row>
     <row r="346" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A346" s="2" t="s">
-        <v>710</v>
+      <c r="A346" t="s">
+        <v>612</v>
       </c>
       <c r="B346" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="C346" t="s">
-        <v>489</v>
+        <v>507</v>
       </c>
       <c r="D346" t="s">
-        <v>484</v>
+        <v>33</v>
+      </c>
+      <c r="E346" s="2">
+        <v>1</v>
       </c>
       <c r="F346" t="s">
         <v>700</v>
@@ -9413,7 +9455,7 @@
     </row>
     <row r="347" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A347" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B347" t="s">
         <v>689</v>
@@ -9424,13 +9466,16 @@
       <c r="D347" t="s">
         <v>484</v>
       </c>
+      <c r="E347" s="2">
+        <v>5</v>
+      </c>
       <c r="F347" t="s">
         <v>700</v>
       </c>
     </row>
     <row r="348" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A348" t="s">
-        <v>615</v>
+      <c r="A348" s="2" t="s">
+        <v>712</v>
       </c>
       <c r="B348" t="s">
         <v>689</v>
@@ -9441,22 +9486,28 @@
       <c r="D348" t="s">
         <v>484</v>
       </c>
+      <c r="E348" s="2">
+        <v>5</v>
+      </c>
       <c r="F348" t="s">
         <v>700</v>
       </c>
     </row>
     <row r="349" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A349" s="2" t="s">
-        <v>711</v>
+      <c r="A349" t="s">
+        <v>614</v>
       </c>
       <c r="B349" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="C349" t="s">
-        <v>507</v>
+        <v>489</v>
       </c>
       <c r="D349" t="s">
-        <v>33</v>
+        <v>484</v>
+      </c>
+      <c r="E349" s="2">
+        <v>5</v>
       </c>
       <c r="F349" t="s">
         <v>700</v>
@@ -9464,81 +9515,87 @@
     </row>
     <row r="350" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A350" t="s">
-        <v>610</v>
+        <v>615</v>
       </c>
       <c r="B350" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="C350" t="s">
-        <v>507</v>
+        <v>489</v>
       </c>
       <c r="D350" t="s">
-        <v>33</v>
+        <v>484</v>
+      </c>
+      <c r="E350" s="2">
+        <v>5</v>
       </c>
       <c r="F350" t="s">
         <v>700</v>
       </c>
     </row>
     <row r="351" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A351" t="s">
-        <v>600</v>
+      <c r="A351" s="2" t="s">
+        <v>711</v>
       </c>
       <c r="B351" t="s">
-        <v>600</v>
+        <v>687</v>
       </c>
       <c r="C351" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="D351" t="s">
-        <v>484</v>
+        <v>33</v>
+      </c>
+      <c r="E351" s="2">
+        <v>1</v>
       </c>
       <c r="F351" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
     </row>
     <row r="352" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A352" t="s">
-        <v>29</v>
-      </c>
-      <c r="B352" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="C352" s="2" t="s">
-        <v>488</v>
-      </c>
-      <c r="D352" s="2" t="s">
-        <v>484</v>
+        <v>610</v>
+      </c>
+      <c r="B352" t="s">
+        <v>687</v>
+      </c>
+      <c r="C352" t="s">
+        <v>507</v>
+      </c>
+      <c r="D352" t="s">
+        <v>33</v>
       </c>
       <c r="E352" s="2">
-        <v>5</v>
-      </c>
-      <c r="F352" s="2" t="s">
-        <v>474</v>
+        <v>1</v>
+      </c>
+      <c r="F352" t="s">
+        <v>700</v>
       </c>
     </row>
     <row r="353" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A353" t="s">
-        <v>30</v>
-      </c>
-      <c r="B353" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="C353" s="2" t="s">
-        <v>488</v>
-      </c>
-      <c r="D353" s="2" t="s">
+        <v>600</v>
+      </c>
+      <c r="B353" t="s">
+        <v>600</v>
+      </c>
+      <c r="C353" t="s">
+        <v>506</v>
+      </c>
+      <c r="D353" t="s">
         <v>484</v>
       </c>
       <c r="E353" s="2">
         <v>5</v>
       </c>
-      <c r="F353" s="2" t="s">
-        <v>474</v>
+      <c r="F353" t="s">
+        <v>702</v>
       </c>
     </row>
     <row r="354" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A354" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B354" s="2" t="s">
         <v>366</v>
@@ -9558,19 +9615,19 @@
     </row>
     <row r="355" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A355" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B355" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C355" s="2" t="s">
-        <v>507</v>
+        <v>488</v>
       </c>
       <c r="D355" s="2" t="s">
-        <v>33</v>
+        <v>484</v>
       </c>
       <c r="E355" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F355" s="2" t="s">
         <v>474</v>
@@ -9578,13 +9635,13 @@
     </row>
     <row r="356" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A356" t="s">
-        <v>266</v>
+        <v>31</v>
       </c>
       <c r="B356" s="2" t="s">
-        <v>422</v>
+        <v>366</v>
       </c>
       <c r="C356" s="2" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D356" s="2" t="s">
         <v>484</v>
@@ -9598,19 +9655,19 @@
     </row>
     <row r="357" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A357" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B357" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C357" s="2" t="s">
-        <v>487</v>
+        <v>507</v>
       </c>
       <c r="D357" s="2" t="s">
-        <v>484</v>
+        <v>33</v>
       </c>
       <c r="E357" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F357" s="2" t="s">
         <v>474</v>
@@ -9618,10 +9675,10 @@
     </row>
     <row r="358" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A358" t="s">
-        <v>35</v>
+        <v>266</v>
       </c>
       <c r="B358" s="2" t="s">
-        <v>368</v>
+        <v>422</v>
       </c>
       <c r="C358" s="2" t="s">
         <v>487</v>
@@ -9638,7 +9695,7 @@
     </row>
     <row r="359" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A359" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B359" s="2" t="s">
         <v>368</v>
@@ -9658,7 +9715,7 @@
     </row>
     <row r="360" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A360" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B360" s="2" t="s">
         <v>368</v>
@@ -9677,11 +9734,11 @@
       </c>
     </row>
     <row r="361" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A361" s="2" t="s">
-        <v>712</v>
+      <c r="A361" t="s">
+        <v>36</v>
       </c>
       <c r="B361" s="2" t="s">
-        <v>713</v>
+        <v>368</v>
       </c>
       <c r="C361" s="2" t="s">
         <v>487</v>
@@ -9698,7 +9755,7 @@
     </row>
     <row r="362" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A362" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B362" s="2" t="s">
         <v>368</v>
@@ -9717,11 +9774,11 @@
       </c>
     </row>
     <row r="363" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A363" t="s">
-        <v>39</v>
+      <c r="A363" s="2" t="s">
+        <v>724</v>
       </c>
       <c r="B363" s="2" t="s">
-        <v>368</v>
+        <v>725</v>
       </c>
       <c r="C363" s="2" t="s">
         <v>487</v>
@@ -9738,7 +9795,7 @@
     </row>
     <row r="364" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A364" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="B364" s="2" t="s">
         <v>368</v>
@@ -9758,7 +9815,7 @@
     </row>
     <row r="365" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A365" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="B365" s="2" t="s">
         <v>368</v>
@@ -9778,19 +9835,19 @@
     </row>
     <row r="366" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A366" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="B366" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C366" s="2" t="s">
-        <v>506</v>
+        <v>487</v>
       </c>
       <c r="D366" s="2" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="E366" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F366" s="2" t="s">
         <v>474</v>
@@ -9798,10 +9855,10 @@
     </row>
     <row r="367" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A367" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="B367" s="2" t="s">
-        <v>470</v>
+        <v>368</v>
       </c>
       <c r="C367" s="2" t="s">
         <v>487</v>
@@ -9817,31 +9874,31 @@
       </c>
     </row>
     <row r="368" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A368" s="2" t="s">
-        <v>715</v>
+      <c r="A368" t="s">
+        <v>40</v>
       </c>
       <c r="B368" s="2" t="s">
-        <v>470</v>
+        <v>369</v>
       </c>
       <c r="C368" s="2" t="s">
-        <v>487</v>
+        <v>506</v>
       </c>
       <c r="D368" s="2" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E368" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F368" s="2" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="369" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A369" s="2" t="s">
-        <v>716</v>
+      <c r="A369" t="s">
+        <v>43</v>
       </c>
       <c r="B369" s="2" t="s">
-        <v>368</v>
+        <v>470</v>
       </c>
       <c r="C369" s="2" t="s">
         <v>487</v>
@@ -9857,8 +9914,8 @@
       </c>
     </row>
     <row r="370" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A370" t="s">
-        <v>44</v>
+      <c r="A370" s="2" t="s">
+        <v>726</v>
       </c>
       <c r="B370" s="2" t="s">
         <v>470</v>
@@ -9877,11 +9934,11 @@
       </c>
     </row>
     <row r="371" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A371" t="s">
-        <v>45</v>
+      <c r="A371" s="2" t="s">
+        <v>727</v>
       </c>
       <c r="B371" s="2" t="s">
-        <v>470</v>
+        <v>368</v>
       </c>
       <c r="C371" s="2" t="s">
         <v>487</v>
@@ -9898,7 +9955,7 @@
     </row>
     <row r="372" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A372" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B372" s="2" t="s">
         <v>470</v>
@@ -9918,7 +9975,7 @@
     </row>
     <row r="373" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A373" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="B373" s="2" t="s">
         <v>470</v>
@@ -9938,19 +9995,19 @@
     </row>
     <row r="374" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A374" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B374" s="2" t="s">
-        <v>698</v>
+        <v>470</v>
       </c>
       <c r="C374" s="2" t="s">
-        <v>506</v>
+        <v>487</v>
       </c>
       <c r="D374" s="2" t="s">
-        <v>33</v>
+        <v>484</v>
       </c>
       <c r="E374" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F374" s="2" t="s">
         <v>474</v>
@@ -9958,19 +10015,19 @@
     </row>
     <row r="375" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A375" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="B375" s="2" t="s">
-        <v>698</v>
+        <v>470</v>
       </c>
       <c r="C375" s="2" t="s">
-        <v>506</v>
+        <v>487</v>
       </c>
       <c r="D375" s="2" t="s">
-        <v>33</v>
+        <v>484</v>
       </c>
       <c r="E375" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F375" s="2" t="s">
         <v>474</v>
@@ -9978,19 +10035,19 @@
     </row>
     <row r="376" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A376" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B376" s="2" t="s">
-        <v>370</v>
+        <v>698</v>
       </c>
       <c r="C376" s="2" t="s">
-        <v>488</v>
+        <v>506</v>
       </c>
       <c r="D376" s="2" t="s">
-        <v>484</v>
+        <v>33</v>
       </c>
       <c r="E376" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F376" s="2" t="s">
         <v>474</v>
@@ -9998,27 +10055,27 @@
     </row>
     <row r="377" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A377" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B377" s="2" t="s">
-        <v>370</v>
+        <v>698</v>
       </c>
       <c r="C377" s="2" t="s">
-        <v>488</v>
+        <v>506</v>
       </c>
       <c r="D377" s="2" t="s">
-        <v>484</v>
+        <v>33</v>
       </c>
       <c r="E377" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F377" s="2" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="378" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A378" s="2" t="s">
-        <v>740</v>
+      <c r="A378" t="s">
+        <v>47</v>
       </c>
       <c r="B378" s="2" t="s">
         <v>370</v>
@@ -10038,7 +10095,7 @@
     </row>
     <row r="379" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A379" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B379" s="2" t="s">
         <v>370</v>
@@ -10057,8 +10114,8 @@
       </c>
     </row>
     <row r="380" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A380" t="s">
-        <v>50</v>
+      <c r="A380" s="2" t="s">
+        <v>728</v>
       </c>
       <c r="B380" s="2" t="s">
         <v>370</v>
@@ -10078,7 +10135,7 @@
     </row>
     <row r="381" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A381" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B381" s="2" t="s">
         <v>370</v>
@@ -10090,7 +10147,7 @@
         <v>484</v>
       </c>
       <c r="E381" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F381" s="2" t="s">
         <v>474</v>
@@ -10098,7 +10155,7 @@
     </row>
     <row r="382" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A382" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B382" s="2" t="s">
         <v>370</v>
@@ -10118,7 +10175,7 @@
     </row>
     <row r="383" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A383" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="B383" s="2" t="s">
         <v>370</v>
@@ -10130,7 +10187,7 @@
         <v>484</v>
       </c>
       <c r="E383" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F383" s="2" t="s">
         <v>474</v>
@@ -10138,13 +10195,13 @@
     </row>
     <row r="384" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A384" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="B384" s="2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C384" s="2" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="D384" s="2" t="s">
         <v>484</v>
@@ -10158,13 +10215,13 @@
     </row>
     <row r="385" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A385" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="B385" s="2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C385" s="2" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="D385" s="2" t="s">
         <v>484</v>
@@ -10178,7 +10235,7 @@
     </row>
     <row r="386" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A386" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B386" s="2" t="s">
         <v>371</v>
@@ -10198,7 +10255,7 @@
     </row>
     <row r="387" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A387" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B387" s="2" t="s">
         <v>371</v>
@@ -10218,7 +10275,7 @@
     </row>
     <row r="388" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A388" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B388" s="2" t="s">
         <v>371</v>
@@ -10238,7 +10295,7 @@
     </row>
     <row r="389" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A389" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B389" s="2" t="s">
         <v>371</v>
@@ -10258,50 +10315,56 @@
     </row>
     <row r="390" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A390" t="s">
-        <v>616</v>
-      </c>
-      <c r="B390" t="s">
-        <v>703</v>
-      </c>
-      <c r="C390" t="s">
-        <v>506</v>
-      </c>
-      <c r="D390" t="s">
-        <v>484</v>
-      </c>
-      <c r="F390" t="s">
+        <v>56</v>
+      </c>
+      <c r="B390" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="C390" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="D390" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="E390" s="2">
+        <v>5</v>
+      </c>
+      <c r="F390" s="2" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="391" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A391" t="s">
-        <v>529</v>
+        <v>62</v>
       </c>
       <c r="B391" s="2" t="s">
-        <v>669</v>
-      </c>
-      <c r="C391" t="s">
-        <v>506</v>
-      </c>
-      <c r="D391" t="s">
-        <v>484</v>
-      </c>
-      <c r="F391" t="s">
+        <v>371</v>
+      </c>
+      <c r="C391" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="D391" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="E391" s="2">
+        <v>5</v>
+      </c>
+      <c r="F391" s="2" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="392" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A392" t="s">
-        <v>531</v>
-      </c>
-      <c r="B392" s="2" t="s">
-        <v>671</v>
+        <v>616</v>
+      </c>
+      <c r="B392" t="s">
+        <v>703</v>
       </c>
       <c r="C392" t="s">
         <v>506</v>
       </c>
       <c r="D392" t="s">
-        <v>33</v>
+        <v>484</v>
       </c>
       <c r="F392" t="s">
         <v>474</v>
@@ -10309,10 +10372,10 @@
     </row>
     <row r="393" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A393" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B393" s="2" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="C393" t="s">
         <v>506</v>
@@ -10326,10 +10389,10 @@
     </row>
     <row r="394" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A394" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B394" s="2" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="C394" t="s">
         <v>506</v>
@@ -10343,59 +10406,53 @@
     </row>
     <row r="395" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A395" t="s">
-        <v>268</v>
+        <v>530</v>
       </c>
       <c r="B395" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="C395" s="2" t="s">
-        <v>668</v>
-      </c>
-      <c r="D395" s="2" t="s">
-        <v>483</v>
-      </c>
-      <c r="E395" s="2">
-        <v>3</v>
-      </c>
-      <c r="F395" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="C395" t="s">
+        <v>506</v>
+      </c>
+      <c r="D395" t="s">
+        <v>484</v>
+      </c>
+      <c r="F395" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="396" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A396" t="s">
-        <v>125</v>
+        <v>532</v>
       </c>
       <c r="B396" s="2" t="s">
-        <v>379</v>
-      </c>
-      <c r="C396" s="2" t="s">
-        <v>668</v>
-      </c>
-      <c r="D396" s="2" t="s">
-        <v>484</v>
-      </c>
-      <c r="E396" s="2">
-        <v>5</v>
-      </c>
-      <c r="F396" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="C396" t="s">
+        <v>506</v>
+      </c>
+      <c r="D396" t="s">
+        <v>33</v>
+      </c>
+      <c r="F396" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="397" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A397" t="s">
-        <v>126</v>
+        <v>268</v>
       </c>
       <c r="B397" s="2" t="s">
-        <v>379</v>
+        <v>423</v>
       </c>
       <c r="C397" s="2" t="s">
         <v>668</v>
       </c>
       <c r="D397" s="2" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="E397" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F397" s="2" t="s">
         <v>474</v>
@@ -10403,13 +10460,13 @@
     </row>
     <row r="398" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A398" t="s">
-        <v>269</v>
+        <v>125</v>
       </c>
       <c r="B398" s="2" t="s">
-        <v>424</v>
+        <v>379</v>
       </c>
       <c r="C398" s="2" t="s">
-        <v>490</v>
+        <v>668</v>
       </c>
       <c r="D398" s="2" t="s">
         <v>484</v>
@@ -10423,13 +10480,13 @@
     </row>
     <row r="399" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A399" t="s">
-        <v>179</v>
+        <v>126</v>
       </c>
       <c r="B399" s="2" t="s">
-        <v>394</v>
+        <v>379</v>
       </c>
       <c r="C399" s="2" t="s">
-        <v>490</v>
+        <v>668</v>
       </c>
       <c r="D399" s="2" t="s">
         <v>484</v>
@@ -10443,13 +10500,13 @@
     </row>
     <row r="400" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A400" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B400" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C400" s="2" t="s">
-        <v>506</v>
+        <v>490</v>
       </c>
       <c r="D400" s="2" t="s">
         <v>484</v>
@@ -10463,19 +10520,19 @@
     </row>
     <row r="401" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A401" t="s">
-        <v>271</v>
+        <v>179</v>
       </c>
       <c r="B401" s="2" t="s">
-        <v>426</v>
+        <v>394</v>
       </c>
       <c r="C401" s="2" t="s">
-        <v>506</v>
+        <v>490</v>
       </c>
       <c r="D401" s="2" t="s">
-        <v>33</v>
+        <v>484</v>
       </c>
       <c r="E401" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F401" s="2" t="s">
         <v>474</v>
@@ -10483,13 +10540,13 @@
     </row>
     <row r="402" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A402" t="s">
-        <v>219</v>
+        <v>270</v>
       </c>
       <c r="B402" s="2" t="s">
-        <v>406</v>
+        <v>425</v>
       </c>
       <c r="C402" s="2" t="s">
-        <v>490</v>
+        <v>506</v>
       </c>
       <c r="D402" s="2" t="s">
         <v>484</v>
@@ -10502,20 +10559,20 @@
       </c>
     </row>
     <row r="403" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A403" s="2" t="s">
-        <v>730</v>
+      <c r="A403" t="s">
+        <v>271</v>
       </c>
       <c r="B403" s="2" t="s">
-        <v>406</v>
+        <v>426</v>
       </c>
       <c r="C403" s="2" t="s">
-        <v>490</v>
+        <v>506</v>
       </c>
       <c r="D403" s="2" t="s">
-        <v>484</v>
+        <v>33</v>
       </c>
       <c r="E403" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F403" s="2" t="s">
         <v>474</v>
@@ -10523,7 +10580,7 @@
     </row>
     <row r="404" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A404" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B404" s="2" t="s">
         <v>406</v>
@@ -10542,20 +10599,20 @@
       </c>
     </row>
     <row r="405" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A405" t="s">
-        <v>272</v>
+      <c r="A405" s="2" t="s">
+        <v>729</v>
       </c>
       <c r="B405" s="2" t="s">
-        <v>427</v>
+        <v>406</v>
       </c>
       <c r="C405" s="2" t="s">
-        <v>506</v>
+        <v>490</v>
       </c>
       <c r="D405" s="2" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="E405" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F405" s="2" t="s">
         <v>474</v>
@@ -10563,19 +10620,19 @@
     </row>
     <row r="406" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A406" t="s">
-        <v>273</v>
+        <v>220</v>
       </c>
       <c r="B406" s="2" t="s">
-        <v>427</v>
+        <v>406</v>
       </c>
       <c r="C406" s="2" t="s">
-        <v>506</v>
+        <v>490</v>
       </c>
       <c r="D406" s="2" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="E406" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F406" s="2" t="s">
         <v>474</v>
@@ -10583,7 +10640,7 @@
     </row>
     <row r="407" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A407" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B407" s="2" t="s">
         <v>427</v>
@@ -10603,104 +10660,104 @@
     </row>
     <row r="408" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A408" t="s">
-        <v>617</v>
-      </c>
-      <c r="B408" t="s">
-        <v>690</v>
-      </c>
-      <c r="C408" t="s">
-        <v>507</v>
-      </c>
-      <c r="D408" t="s">
-        <v>33</v>
-      </c>
-      <c r="F408" t="s">
+        <v>273</v>
+      </c>
+      <c r="B408" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="C408" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="D408" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="E408" s="2">
+        <v>2</v>
+      </c>
+      <c r="F408" s="2" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="409" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A409" s="2" t="s">
-        <v>714</v>
-      </c>
-      <c r="B409" t="s">
-        <v>434</v>
-      </c>
-      <c r="C409" t="s">
-        <v>487</v>
-      </c>
-      <c r="D409" t="s">
-        <v>484</v>
-      </c>
-      <c r="E409">
-        <v>5</v>
-      </c>
-      <c r="F409" t="s">
+      <c r="A409" t="s">
+        <v>274</v>
+      </c>
+      <c r="B409" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="C409" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="D409" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="E409" s="2">
+        <v>2</v>
+      </c>
+      <c r="F409" s="2" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="410" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A410" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B410" t="s">
-        <v>434</v>
+        <v>690</v>
       </c>
       <c r="C410" t="s">
-        <v>487</v>
+        <v>507</v>
       </c>
       <c r="D410" t="s">
-        <v>484</v>
-      </c>
-      <c r="E410">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="F410" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="411" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A411" t="s">
+      <c r="A411" s="2" t="s">
+        <v>730</v>
+      </c>
+      <c r="B411" t="s">
+        <v>434</v>
+      </c>
+      <c r="C411" t="s">
+        <v>487</v>
+      </c>
+      <c r="D411" t="s">
+        <v>484</v>
+      </c>
+      <c r="E411">
+        <v>5</v>
+      </c>
+      <c r="F411" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="412" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A412" t="s">
+        <v>618</v>
+      </c>
+      <c r="B412" t="s">
+        <v>434</v>
+      </c>
+      <c r="C412" t="s">
+        <v>487</v>
+      </c>
+      <c r="D412" t="s">
+        <v>484</v>
+      </c>
+      <c r="E412">
+        <v>5</v>
+      </c>
+      <c r="F412" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="413" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A413" t="s">
         <v>284</v>
-      </c>
-      <c r="B411" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="C411" s="2" t="s">
-        <v>487</v>
-      </c>
-      <c r="D411" s="2" t="s">
-        <v>484</v>
-      </c>
-      <c r="E411" s="2">
-        <v>5</v>
-      </c>
-      <c r="F411" s="2" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="412" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A412" s="2" t="s">
-        <v>714</v>
-      </c>
-      <c r="B412" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="C412" s="2" t="s">
-        <v>487</v>
-      </c>
-      <c r="D412" s="2" t="s">
-        <v>484</v>
-      </c>
-      <c r="E412" s="2">
-        <v>5</v>
-      </c>
-      <c r="F412" s="2" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="413" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A413" s="2" t="s">
-        <v>730</v>
       </c>
       <c r="B413" s="2" t="s">
         <v>434</v>
@@ -10720,7 +10777,7 @@
     </row>
     <row r="414" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A414" s="2" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="B414" s="2" t="s">
         <v>436</v>
@@ -10880,7 +10937,7 @@
     </row>
     <row r="422" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A422" s="2" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="B422" t="s">
         <v>686</v>
@@ -10980,10 +11037,10 @@
     </row>
     <row r="427" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A427" s="2" t="s">
-        <v>722</v>
+        <v>733</v>
       </c>
       <c r="B427" s="2" t="s">
-        <v>723</v>
+        <v>734</v>
       </c>
       <c r="C427" t="s">
         <v>507</v>
@@ -11000,10 +11057,10 @@
     </row>
     <row r="428" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A428" s="2" t="s">
-        <v>727</v>
+        <v>735</v>
       </c>
       <c r="B428" s="2" t="s">
-        <v>724</v>
+        <v>736</v>
       </c>
       <c r="C428" t="s">
         <v>507</v>
@@ -11023,7 +11080,7 @@
         <v>512</v>
       </c>
       <c r="B429" s="2" t="s">
-        <v>726</v>
+        <v>737</v>
       </c>
       <c r="C429" t="s">
         <v>507</v>
@@ -11043,7 +11100,7 @@
         <v>513</v>
       </c>
       <c r="B430" s="2" t="s">
-        <v>725</v>
+        <v>738</v>
       </c>
       <c r="C430" t="s">
         <v>507</v>
@@ -11060,10 +11117,10 @@
     </row>
     <row r="431" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A431" s="2" t="s">
-        <v>720</v>
+        <v>739</v>
       </c>
       <c r="B431" s="2" t="s">
-        <v>721</v>
+        <v>740</v>
       </c>
       <c r="C431" s="2" t="s">
         <v>488</v>
@@ -11120,7 +11177,7 @@
     </row>
     <row r="434" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A434" s="2" t="s">
-        <v>751</v>
+        <v>741</v>
       </c>
       <c r="B434" t="s">
         <v>682</v>
@@ -11140,7 +11197,7 @@
     </row>
     <row r="435" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A435" s="2" t="s">
-        <v>752</v>
+        <v>742</v>
       </c>
       <c r="B435" t="s">
         <v>682</v>
@@ -11160,7 +11217,7 @@
     </row>
     <row r="436" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A436" s="2" t="s">
-        <v>753</v>
+        <v>743</v>
       </c>
       <c r="B436" t="s">
         <v>682</v>
@@ -11180,7 +11237,7 @@
     </row>
     <row r="437" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A437" s="2" t="s">
-        <v>754</v>
+        <v>744</v>
       </c>
       <c r="B437" t="s">
         <v>682</v>
@@ -11200,7 +11257,7 @@
     </row>
     <row r="438" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A438" s="2" t="s">
-        <v>755</v>
+        <v>745</v>
       </c>
       <c r="B438" t="s">
         <v>684</v>
@@ -11220,7 +11277,7 @@
     </row>
     <row r="439" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A439" s="2" t="s">
-        <v>756</v>
+        <v>746</v>
       </c>
       <c r="B439" t="s">
         <v>684</v>
@@ -11240,7 +11297,7 @@
     </row>
     <row r="440" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A440" s="2" t="s">
-        <v>757</v>
+        <v>747</v>
       </c>
       <c r="B440" t="s">
         <v>684</v>
@@ -11260,7 +11317,7 @@
     </row>
     <row r="441" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A441" s="2" t="s">
-        <v>758</v>
+        <v>748</v>
       </c>
       <c r="B441" t="s">
         <v>684</v>
@@ -11580,7 +11637,7 @@
     </row>
     <row r="457" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A457" s="2" t="s">
-        <v>738</v>
+        <v>749</v>
       </c>
       <c r="B457" s="2" t="s">
         <v>389</v>
@@ -11780,7 +11837,7 @@
     </row>
     <row r="467" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A467" s="2" t="s">
-        <v>717</v>
+        <v>750</v>
       </c>
       <c r="B467" s="2" t="s">
         <v>448</v>
@@ -12060,10 +12117,10 @@
     </row>
     <row r="481" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A481" s="2" t="s">
-        <v>759</v>
+        <v>751</v>
       </c>
       <c r="B481" s="2" t="s">
-        <v>761</v>
+        <v>752</v>
       </c>
       <c r="C481" t="s">
         <v>488</v>
@@ -12080,10 +12137,10 @@
     </row>
     <row r="482" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A482" s="2" t="s">
-        <v>760</v>
+        <v>753</v>
       </c>
       <c r="B482" s="2" t="s">
-        <v>761</v>
+        <v>752</v>
       </c>
       <c r="C482" t="s">
         <v>488</v>
@@ -13249,10 +13306,10 @@
     </row>
     <row r="543" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A543" s="2" t="s">
-        <v>763</v>
+        <v>754</v>
       </c>
       <c r="B543" s="2" t="s">
-        <v>762</v>
+        <v>755</v>
       </c>
       <c r="C543" s="2" t="s">
         <v>489</v>
@@ -13529,7 +13586,7 @@
     </row>
     <row r="557" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A557" s="2" t="s">
-        <v>741</v>
+        <v>756</v>
       </c>
       <c r="B557" s="2" t="s">
         <v>401</v>
@@ -13549,7 +13606,7 @@
     </row>
     <row r="558" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A558" s="2" t="s">
-        <v>750</v>
+        <v>757</v>
       </c>
       <c r="B558" s="2" t="s">
         <v>401</v>
@@ -13569,7 +13626,7 @@
     </row>
     <row r="559" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A559" s="2" t="s">
-        <v>742</v>
+        <v>758</v>
       </c>
       <c r="B559" s="2" t="s">
         <v>401</v>
@@ -13589,7 +13646,7 @@
     </row>
     <row r="560" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A560" s="2" t="s">
-        <v>743</v>
+        <v>759</v>
       </c>
       <c r="B560" s="2" t="s">
         <v>401</v>
@@ -13609,7 +13666,7 @@
     </row>
     <row r="561" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A561" s="2" t="s">
-        <v>745</v>
+        <v>760</v>
       </c>
       <c r="B561" s="2" t="s">
         <v>401</v>
@@ -13629,7 +13686,7 @@
     </row>
     <row r="562" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A562" s="2" t="s">
-        <v>746</v>
+        <v>761</v>
       </c>
       <c r="B562" s="2" t="s">
         <v>692</v>
@@ -13649,7 +13706,7 @@
     </row>
     <row r="563" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A563" s="2" t="s">
-        <v>749</v>
+        <v>762</v>
       </c>
       <c r="B563" s="2" t="s">
         <v>692</v>
@@ -13669,10 +13726,10 @@
     </row>
     <row r="564" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A564" s="2" t="s">
-        <v>747</v>
+        <v>763</v>
       </c>
       <c r="B564" s="2" t="s">
-        <v>748</v>
+        <v>764</v>
       </c>
       <c r="C564" s="2" t="s">
         <v>487</v>
@@ -13688,7 +13745,11 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F556" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:F522" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F522">
+      <sortCondition ref="F1:F520"/>
+    </sortState>
+  </autoFilter>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>